<commit_message>
feat: Migration 032 - Nettoyage codes et localités sondages
- Remplir code depuis meta->>'code' (123 sondages)
- Remplir localite_base depuis meta->>'localite' (123 sondages)
- Générer localite_key normalisée (UPPER + sans accents)
- Ajouter contrainte NOT NULL sur code
- Créer index sur localite_key
- Fix erreur 500 sur /sondages?missing=geom

Tous les sondages ont maintenant un code valide et une localité.
</commit_message>
<xml_diff>
--- a/data/xlsx/Granulométrie.xlsx
+++ b/data/xlsx/Granulométrie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO T470\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJET_ATLAS_MASTER\atlas\data\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BB924E-FEB0-491B-9D89-DF8C2B26992F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F2447D-84C1-449B-8E4E-6A6B8D1DD551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" activeTab="5" xr2:uid="{334D33F4-E8A1-4F20-9E6E-D82714B401DC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{334D33F4-E8A1-4F20-9E6E-D82714B401DC}"/>
   </bookViews>
   <sheets>
     <sheet name="3.1" sheetId="1" r:id="rId1"/>
@@ -619,13 +619,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C64B15D-2201-481E-8945-01CE347190D3}">
   <dimension ref="B4:F16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.90625" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -642,7 +642,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>1</v>
       </c>
@@ -659,7 +659,7 @@
         <v>74.849999999999994</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>2</v>
       </c>
@@ -676,7 +676,7 @@
         <v>47.15</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>3</v>
       </c>
@@ -693,7 +693,7 @@
         <v>32.25</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -710,7 +710,7 @@
         <v>63.99</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -727,7 +727,7 @@
         <v>38.18</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>6</v>
       </c>
@@ -744,7 +744,7 @@
         <v>62.96</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>7</v>
       </c>
@@ -761,7 +761,7 @@
         <v>74.87</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>8</v>
       </c>
@@ -778,7 +778,7 @@
         <v>72.66</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>9</v>
       </c>
@@ -792,7 +792,7 @@
         <v>54.5</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>10</v>
       </c>
@@ -809,7 +809,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>11</v>
       </c>
@@ -826,7 +826,7 @@
         <v>53.52</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>12</v>
       </c>
@@ -851,12 +851,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{157D8EFE-520D-4326-BAE5-505494DDD527}">
   <dimension ref="A2:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -873,7 +873,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -890,7 +890,7 @@
         <v>33.44</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -907,7 +907,7 @@
         <v>24.02</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -924,7 +924,7 @@
         <v>43.17</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -941,7 +941,7 @@
         <v>36.659999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -958,7 +958,7 @@
         <v>44.24</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -975,7 +975,7 @@
         <v>48.1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -992,7 +992,7 @@
         <v>53.44</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -1017,12 +1017,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E43C1FA8-C1A3-4835-AF70-E878FA368EA7}">
   <dimension ref="B4:F22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>1</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>42.8</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>2</v>
       </c>
@@ -1073,7 +1073,7 @@
         <v>30.07</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>3</v>
       </c>
@@ -1090,7 +1090,7 @@
         <v>63.99</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>42.25</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>67.3</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>6</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>61.54</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>7</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>53.84</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>8</v>
       </c>
@@ -1172,7 +1172,7 @@
         <v>40.1</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>9</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>38.18</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>10</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>42.63</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>11</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>80.58</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>12</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>56.37</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>13</v>
       </c>
@@ -1257,7 +1257,7 @@
         <v>64.319999999999993</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>14</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>74.150000000000006</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>15</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>53.1</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>16</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>66.42</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>17</v>
       </c>
@@ -1325,7 +1325,7 @@
         <v>74.73</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>18</v>
       </c>
@@ -1350,12 +1350,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75118E9B-C346-4495-AC79-AC0771268F88}">
   <dimension ref="B4:F14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -1372,7 +1372,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>1</v>
       </c>
@@ -1389,7 +1389,7 @@
         <v>63.34</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>2</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>33.049999999999997</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>3</v>
       </c>
@@ -1423,7 +1423,7 @@
         <v>41.83</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>4</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>56.61</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>5</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>28.89</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>6</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>49.9</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>7</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>53.41</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>8</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>55.25</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>9</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>32.340000000000003</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>10</v>
       </c>
@@ -1550,12 +1550,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11AC969D-88AE-4A7F-BD2F-B783704E0D32}">
   <dimension ref="B5:F16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>52.58</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>2</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>53.47</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>3</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>24.53</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>4</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>32.270000000000003</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>5</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>51.26</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>6</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>67.3</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>7</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>53.84</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>8</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>65.5</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>9</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>65.12</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>10</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>65.55</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>11</v>
       </c>
@@ -1767,12 +1767,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44A152AE-1877-44E9-84E2-D0E9FC9BFFE9}">
   <dimension ref="B5:F22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="18.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>1</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>57.81</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7">
         <v>2</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>51.27</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>3</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>64.81</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>4</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>33.299999999999997</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10">
         <v>5</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>58.88</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>6</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>39.89</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>7</v>
       </c>
@@ -1908,7 +1908,7 @@
         <v>44.56</v>
       </c>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B13">
         <v>8</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>36.130000000000003</v>
       </c>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B14">
         <v>9</v>
       </c>
@@ -1942,7 +1942,7 @@
         <v>21.78</v>
       </c>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B15">
         <v>10</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>41.68</v>
       </c>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B16">
         <v>11</v>
       </c>
@@ -1976,7 +1976,7 @@
         <v>44.6</v>
       </c>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>12</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>58.75</v>
       </c>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>13</v>
       </c>
@@ -2010,7 +2010,7 @@
         <v>33.21</v>
       </c>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>14</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>54.01</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>15</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>57.8</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>16</v>
       </c>
@@ -2061,7 +2061,10 @@
         <v>58.36</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>17</v>
+      </c>
       <c r="C22" t="s">
         <v>77</v>
       </c>

</xml_diff>